<commit_message>
remove some test files
</commit_message>
<xml_diff>
--- a/20260514_docx_to_markdown/final/fixtures/xlsx/example.xlsx
+++ b/20260514_docx_to_markdown/final/fixtures/xlsx/example.xlsx
@@ -5,17 +5,19 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kazuj\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\home\kazufusa\src\github.com\kazufusa\til\20260514_docx_to_markdown\final\fixtures\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85C65F4D-95DF-4ADA-887C-F52E6EFEAFC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E467BC3-63B5-412E-8FD4-9147FC61F1FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="売上" sheetId="1" r:id="rId1"/>
     <sheet name="photos" sheetId="2" r:id="rId2"/>
     <sheet name="calculation" sheetId="3" r:id="rId3"/>
+    <sheet name="売上一覧" sheetId="4" r:id="rId4"/>
+    <sheet name="構成比" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +41,7 @@
   <metadataTypes count="1">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="2">
+  <futureMetadata name="XLRICHVALUE" count="4">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
@@ -54,20 +56,40 @@
         </ext>
       </extLst>
     </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="2"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="3"/>
+        </ext>
+      </extLst>
+    </bk>
   </futureMetadata>
-  <valueMetadata count="2">
+  <valueMetadata count="4">
     <bk>
       <rc t="1" v="0"/>
     </bk>
     <bk>
       <rc t="1" v="1"/>
     </bk>
+    <bk>
+      <rc t="1" v="2"/>
+    </bk>
+    <bk>
+      <rc t="1" v="3"/>
+    </bk>
   </valueMetadata>
 </metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
   <si>
     <t>Apples</t>
   </si>
@@ -112,6 +134,63 @@
   </si>
   <si>
     <t>avg</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>商品名</t>
+  </si>
+  <si>
+    <t>数量</t>
+  </si>
+  <si>
+    <t>単価</t>
+  </si>
+  <si>
+    <t>合計</t>
+  </si>
+  <si>
+    <t>りんご</t>
+  </si>
+  <si>
+    <t>バナナ</t>
+  </si>
+  <si>
+    <t>みかん</t>
+  </si>
+  <si>
+    <t>区分</t>
+  </si>
+  <si>
+    <t>割合(%)</t>
+  </si>
+  <si>
+    <t>個人</t>
+  </si>
+  <si>
+    <t>法人</t>
+  </si>
+  <si>
+    <t>その他</t>
+  </si>
+  <si>
+    <t>犬1</t>
+    <rPh sb="0" eb="1">
+      <t>イヌ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>犬2</t>
+    <rPh sb="0" eb="1">
+      <t>イヌ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>犬3</t>
+    <rPh sb="0" eb="1">
+      <t>イヌ</t>
+    </rPh>
     <phoneticPr fontId="2"/>
   </si>
 </sst>
@@ -119,7 +198,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -139,6 +218,13 @@
       <family val="3"/>
       <charset val="128"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
     </font>
   </fonts>
   <fills count="2">
@@ -161,7 +247,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -172,6 +258,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -1161,6 +1248,94 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2857500" cy="1714500"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5B8EB3C8-5073-4F27-832D-1AB8B4624EAD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="990600"/>
+          <a:ext cx="2857500" cy="1714500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1016000</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>146050</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2286000" cy="2286000"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D3CC2FA7-D7E5-4878-8076-AD019D6D1A49}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6261100" y="146050"/>
+          <a:ext cx="2286000" cy="2286000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
 <rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
   <global>
@@ -1202,7 +1377,7 @@
 </file>
 
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="2">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="4">
   <rv s="0">
     <v>0</v>
     <v>5</v>
@@ -1211,6 +1386,14 @@
     <v>1</v>
     <v>5</v>
     <v>混雑した通りにいる人</v>
+  </rv>
+  <rv s="0">
+    <v>2</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>3</v>
+    <v>5</v>
   </rv>
 </rvData>
 </file>
@@ -1233,6 +1416,8 @@
 <richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <rel r:id="rId1"/>
   <rel r:id="rId2"/>
+  <rel r:id="rId3"/>
+  <rel r:id="rId4"/>
 </richValueRels>
 </file>
 
@@ -1696,4 +1881,148 @@
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0397F425-533E-4738-8F3D-2A7BA24AA844}">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="3" width="10" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2">
+        <v>3</v>
+      </c>
+      <c r="C2">
+        <v>150</v>
+      </c>
+      <c r="D2">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3">
+        <v>5</v>
+      </c>
+      <c r="C3">
+        <v>100</v>
+      </c>
+      <c r="D3">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4">
+        <v>8</v>
+      </c>
+      <c r="C4">
+        <v>80</v>
+      </c>
+      <c r="D4">
+        <v>640</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEF3D3B7-1A6A-49EA-B508-4564402B3727}">
+  <dimension ref="A1:C18"/>
+  <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="39.7265625" customWidth="1"/>
+    <col min="2" max="2" width="35.36328125" customWidth="1"/>
+    <col min="3" max="3" width="34.7265625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17" t="s">
+        <v>26</v>
+      </c>
+      <c r="C17" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="174" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="B18" t="e" vm="3">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C18" t="e" vm="4">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>